<commit_message>
CAR Mujeres banca: boquilla en lugar de sumidero cupula, sin uniones, un tramo de canaleta de 2.00 m por techo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_mujeres/METRADO_CANALETA_Y_ACCESORIOS_BANCAS_CAR_MUJERES.xlsx
+++ b/entregables_mujeres/METRADO_CANALETA_Y_ACCESORIOS_BANCAS_CAR_MUJERES.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -585,7 +585,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>N.° DE BANCAS (techos iguales)</t>
+          <t>N.° DE TECHOS IGUALES (BANCAS)</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -610,12 +610,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>CANT. POR BANCA</t>
+          <t>METRADO POR TECHO</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>N.° BANCAS</t>
+          <t>N.° DE TECHOS</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Largo del techo de la banca: 2.00 m (planta de techo; corte B-B, lamina DB-03)</t>
+          <t>1 tramo de 2.00 m por techo (techo a una agua, sin uniones de canaleta)</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Una en cada extremo de la canaleta</t>
+          <t>Una en cada extremo del tramo</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>SUMIDERO DE CANALETA TIPO CUPULA 4"</t>
+          <t>BOQUILLA DE PLANCHA DE ALUZINC P/CONEXION DE CANALETA A TUBERIA PVC 4"</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>En el fondo de la canaleta, a 0.30 m del extremo, sobre la bajada</t>
+          <t>Brida 0.16 x 0.16 con 8 remaches y sellador, cuello Ø 0.10 x 0.15; a 0.30 m del extremo</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Bajo el sumidero y sobre la bajada (corte A-A)</t>
+          <t>Bajo la boquilla y sobre la bajada (corte A-A)</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>UNION PVC 4"</t>
+          <t>COLGADOR F°G° C/VARILLA ROSCADA 3/8" P/TUBERIA PVC 4"</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="9">
         <f>$D$8</f>
@@ -823,7 +823,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Bajo el sumidero y bajo el segundo codo (corte A-A)</t>
+          <t>Sobre el tramo horizontal, colgado de la viga metalica 2" x 2"</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>COLGADOR F°G° C/VARILLA ROSCADA 3/8" P/TUBERIA PVC 4"</t>
+          <t>ABRAZADERA DE PLATINA F°G° 1" x 1/8" P/TUBERIA PVC 4"</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -856,47 +856,14 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Sobre el tramo horizontal, colgado de la viga metalica 2" x 2"</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>08</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>ABRAZADERA DE PLATINA F°G° 1" x 1/8" P/TUBERIA PVC 4"</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="9">
-        <f>$D$8</f>
-        <v/>
-      </c>
-      <c r="F18" s="12">
-        <f>D18*E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
           <t>En la bajada, fijada a la columna metalica (+1.77)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>Notas: no incluye el tubo PVC 4" ni la falsa columna. Celda amarilla = dato; celda verde = formula. Cantidades por banca segun el detalle de banca tipo 01 y las laminas DB-01 (isometrico), DB-02 (detalles) y DB-03 (cortes A-A y B-B).</t>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Notas: no incluye el tubo PVC 4" ni la falsa columna. Un solo tramo de canaleta por techo (a una agua), sin uniones. Celda amarilla = dato; celda verde = formula. Cantidades por banca segun el detalle de banca tipo 01 y las laminas DB-01 (isometrico), DB-02 (detalles) y DB-03 (cortes A-A y B-B).</t>
         </is>
       </c>
     </row>
@@ -906,8 +873,8 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B5:G5"/>
     <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A20:G20"/>
     <mergeCell ref="B4:G4"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
CAR Mujeres banca: canaleta, tapas y boquilla de aluzinc e = 0.50 mm en planos y metrado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_mujeres/METRADO_CANALETA_Y_ACCESORIOS_BANCAS_CAR_MUJERES.xlsx
+++ b/entregables_mujeres/METRADO_CANALETA_Y_ACCESORIOS_BANCAS_CAR_MUJERES.xlsx
@@ -637,7 +637,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CANALETA DE PLANCHA DE ALUZINC, SECCION INTERIOR 0.18 m (ANCHO) x 0.20 m (ALTO)</t>
+          <t>CANALETA DE PLANCHA DE ALUZINC e=0.50mm, SECCION INTERIOR 0.18 m (ANCHO) x 0.20 m (ALTO)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>TAPA LATERAL DE ALUZINC P/CANALETA</t>
+          <t>TAPA LATERAL DE PLANCHA DE ALUZINC e=0.50mm P/CANALETA</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>BOQUILLA DE PLANCHA DE ALUZINC P/CONEXION DE CANALETA A TUBERIA PVC 4"</t>
+          <t>BOQUILLA DE PLANCHA DE ALUZINC e=0.50mm P/CONEXION DE CANALETA A TUBERIA PVC 4"</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">

</xml_diff>